<commit_message>
Deploying to gh-pages from @ mattaq31/Hash-CAD@d8396be16fae5ae0edf5166d952e6bf70651e50f 🚀
</commit_message>
<xml_diff>
--- a/plates/cargo_plates/P3518_MA_octahedron_patterning_v1.xlsx
+++ b/plates/cargo_plates/P3518_MA_octahedron_patterning_v1.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="650">
   <si>
     <t>well</t>
   </si>
@@ -1344,6 +1344,66 @@
     <t>CARGO-GoldWireBinder-h2-position_8</t>
   </si>
   <si>
+    <t>CARGO-antiOcta1-h5-position_2</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_3</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_8</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_9</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_14</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_15</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_20</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_21</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_26</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta1-h5-position_27</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_5</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_6</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_11</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_12</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_17</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_18</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_23</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_24</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_29</t>
+  </si>
+  <si>
+    <t>CARGO-antiOcta2-h5-position_30</t>
+  </si>
+  <si>
     <t>TAGCTGTTTCCTAGCTAACTCACATTAATTGGTTTGCGTATTttTCTATACCTTCATACCTACAC</t>
   </si>
   <si>
@@ -1503,6 +1563,66 @@
     <t>TCAACATTAAATGGCGCATCGTAACCGTGCGGAAACCAGGCAttGGTTGATAAAAGCATGACAGGTTGATAATATAGAT</t>
   </si>
   <si>
+    <t>CATAAAGTGGTGAGACGGGCAACAGCTGAGAAAGCGAAAGGAttACGGTTAT</t>
+  </si>
+  <si>
+    <t>TCTGTGGTGGCTCACAATTCCACACAACCGGTCACGCTGCGCttACGGTTAT</t>
+  </si>
+  <si>
+    <t>GACCGTAATCTGTTGGGAAGGGCGATCGAAAAGAGTCTGTCCttACGGTTAT</t>
+  </si>
+  <si>
+    <t>GGAAGATTGCGTCGGATTCTCCGTGGGACTTCTTTGATTAGTttACGGTTAT</t>
+  </si>
+  <si>
+    <t>GATAAAAACGGTCTTTACCCTGACTATTTGGCCAACAGAGATttACGGTTAT</t>
+  </si>
+  <si>
+    <t>TAAGAACTGCAACACTATCATAACCCTCATACGTGGCACAGAttACGGTTAT</t>
+  </si>
+  <si>
+    <t>CCACCCTCACAGACGTTAGTAAATGAATAATATCAAACCCTCttACGGTTAT</t>
+  </si>
+  <si>
+    <t>ACAGTTAATTCAGGAGGTTTAGTACCGCACAGTTGAAAGGAAttACGGTTAT</t>
+  </si>
+  <si>
+    <t>CTTTACAGAGAAGCCCTTTTTAAGAAAACCAGAAGGAGCGGAttACGGTTAT</t>
+  </si>
+  <si>
+    <t>AACCTCCCGTTTTTGTTTAACGTCAAAAGATGGCAATTCATCttACGGTTAT</t>
+  </si>
+  <si>
+    <t>TTTTCGTCTTCAGCGGGGTCATTGCAGGTATAACGTGCTTTCttATAACCGT</t>
+  </si>
+  <si>
+    <t>TTTCTCCGTTGCTGATTGCCGTTCCGGCAGGAGGCCGATTAAttATAACCGT</t>
+  </si>
+  <si>
+    <t>GGCAAGGCATAGGTAAAGATTCAAAAGGCCGCCAGCCATTGCttATAACCGT</t>
+  </si>
+  <si>
+    <t>AATATGCAATAGTAGTAGCATTAACATCACATTTTGACGCTCttATAACCGT</t>
+  </si>
+  <si>
+    <t>ACGAAAGAGCCGAACTGACCAACTTTGACCGAACGAACCACCttATAACCGT</t>
+  </si>
+  <si>
+    <t>CGCCCACGCTACGTAATGCCACTACGAATCAGTATTAACACCttATAACCGT</t>
+  </si>
+  <si>
+    <t>GAATCAAGTCCCTCAGAGCCGCCACCAGACATTTGAGGATTTttATAACCGT</t>
+  </si>
+  <si>
+    <t>CCAAAGACACCATCGATAGCAGCACCGTACAACTCGTATTAAttATAACCGT</t>
+  </si>
+  <si>
+    <t>GTAGGGCTTATAGATAAGTCCTGAACAATTTGCACGTAAAACttATAACCGT</t>
+  </si>
+  <si>
+    <t>ATCGCAAGAAAATTCTTACCAGTATAAAGGTTTAACGTCAGAttATAACCGT</t>
+  </si>
+  <si>
     <t>Cargo Handle For Slat Position 2, Side h2, Cargo ID antiBart</t>
   </si>
   <si>
@@ -1662,6 +1782,66 @@
     <t>Cargo Handle For Slat Position 8, Side h2, Cargo ID GoldWireBinder</t>
   </si>
   <si>
+    <t>Cargo Handle For Slat Position 2, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 3, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 8, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 9, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 14, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 15, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 20, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 21, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 26, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 27, Side h5, Cargo ID antiOcta1</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 5, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 6, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 11, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 12, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 17, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 18, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 23, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 24, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 29, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 30, Side h5, Cargo ID antiOcta2</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -1734,7 +1914,7 @@
     <t>24</t>
   </si>
   <si>
-    <t>P3518_MA_octahedron_patterning_v1</t>
+    <t>P3518_MA_octahedron_patterning_v2_with_octa_handles</t>
   </si>
   <si>
     <t>A</t>
@@ -2199,10 +2379,10 @@
         <v>389</v>
       </c>
       <c r="C2" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="D2" t="s">
-        <v>495</v>
+        <v>535</v>
       </c>
       <c r="E2">
         <v>200</v>
@@ -2216,10 +2396,10 @@
         <v>390</v>
       </c>
       <c r="C3" t="s">
-        <v>443</v>
+        <v>463</v>
       </c>
       <c r="D3" t="s">
-        <v>496</v>
+        <v>536</v>
       </c>
       <c r="E3">
         <v>200</v>
@@ -2233,10 +2413,10 @@
         <v>391</v>
       </c>
       <c r="C4" t="s">
-        <v>444</v>
+        <v>464</v>
       </c>
       <c r="D4" t="s">
-        <v>497</v>
+        <v>537</v>
       </c>
       <c r="E4">
         <v>200</v>
@@ -2250,10 +2430,10 @@
         <v>392</v>
       </c>
       <c r="C5" t="s">
-        <v>445</v>
+        <v>465</v>
       </c>
       <c r="D5" t="s">
-        <v>498</v>
+        <v>538</v>
       </c>
       <c r="E5">
         <v>200</v>
@@ -2267,10 +2447,10 @@
         <v>393</v>
       </c>
       <c r="C6" t="s">
-        <v>446</v>
+        <v>466</v>
       </c>
       <c r="D6" t="s">
-        <v>499</v>
+        <v>539</v>
       </c>
       <c r="E6">
         <v>200</v>
@@ -2284,10 +2464,10 @@
         <v>394</v>
       </c>
       <c r="C7" t="s">
-        <v>447</v>
+        <v>467</v>
       </c>
       <c r="D7" t="s">
-        <v>500</v>
+        <v>540</v>
       </c>
       <c r="E7">
         <v>200</v>
@@ -2301,10 +2481,10 @@
         <v>395</v>
       </c>
       <c r="C8" t="s">
-        <v>448</v>
+        <v>468</v>
       </c>
       <c r="D8" t="s">
-        <v>501</v>
+        <v>541</v>
       </c>
       <c r="E8">
         <v>200</v>
@@ -2318,10 +2498,10 @@
         <v>396</v>
       </c>
       <c r="C9" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="D9" t="s">
-        <v>502</v>
+        <v>542</v>
       </c>
       <c r="E9">
         <v>200</v>
@@ -2335,10 +2515,10 @@
         <v>397</v>
       </c>
       <c r="C10" t="s">
-        <v>450</v>
+        <v>470</v>
       </c>
       <c r="D10" t="s">
-        <v>503</v>
+        <v>543</v>
       </c>
       <c r="E10">
         <v>200</v>
@@ -2352,10 +2532,10 @@
         <v>398</v>
       </c>
       <c r="C11" t="s">
-        <v>451</v>
+        <v>471</v>
       </c>
       <c r="D11" t="s">
-        <v>504</v>
+        <v>544</v>
       </c>
       <c r="E11">
         <v>200</v>
@@ -2439,10 +2619,10 @@
         <v>399</v>
       </c>
       <c r="C26" t="s">
-        <v>452</v>
+        <v>472</v>
       </c>
       <c r="D26" t="s">
-        <v>505</v>
+        <v>545</v>
       </c>
       <c r="E26">
         <v>200</v>
@@ -2456,10 +2636,10 @@
         <v>400</v>
       </c>
       <c r="C27" t="s">
-        <v>453</v>
+        <v>473</v>
       </c>
       <c r="D27" t="s">
-        <v>506</v>
+        <v>546</v>
       </c>
       <c r="E27">
         <v>200</v>
@@ -2473,10 +2653,10 @@
         <v>401</v>
       </c>
       <c r="C28" t="s">
-        <v>454</v>
+        <v>474</v>
       </c>
       <c r="D28" t="s">
-        <v>507</v>
+        <v>547</v>
       </c>
       <c r="E28">
         <v>200</v>
@@ -2490,10 +2670,10 @@
         <v>402</v>
       </c>
       <c r="C29" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="D29" t="s">
-        <v>508</v>
+        <v>548</v>
       </c>
       <c r="E29">
         <v>200</v>
@@ -2507,10 +2687,10 @@
         <v>403</v>
       </c>
       <c r="C30" t="s">
-        <v>456</v>
+        <v>476</v>
       </c>
       <c r="D30" t="s">
-        <v>509</v>
+        <v>549</v>
       </c>
       <c r="E30">
         <v>200</v>
@@ -2524,10 +2704,10 @@
         <v>404</v>
       </c>
       <c r="C31" t="s">
-        <v>457</v>
+        <v>477</v>
       </c>
       <c r="D31" t="s">
-        <v>510</v>
+        <v>550</v>
       </c>
       <c r="E31">
         <v>200</v>
@@ -2541,10 +2721,10 @@
         <v>405</v>
       </c>
       <c r="C32" t="s">
-        <v>458</v>
+        <v>478</v>
       </c>
       <c r="D32" t="s">
-        <v>511</v>
+        <v>551</v>
       </c>
       <c r="E32">
         <v>200</v>
@@ -2558,10 +2738,10 @@
         <v>406</v>
       </c>
       <c r="C33" t="s">
-        <v>459</v>
+        <v>479</v>
       </c>
       <c r="D33" t="s">
-        <v>512</v>
+        <v>552</v>
       </c>
       <c r="E33">
         <v>200</v>
@@ -2575,10 +2755,10 @@
         <v>407</v>
       </c>
       <c r="C34" t="s">
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="D34" t="s">
-        <v>513</v>
+        <v>553</v>
       </c>
       <c r="E34">
         <v>200</v>
@@ -2592,10 +2772,10 @@
         <v>408</v>
       </c>
       <c r="C35" t="s">
-        <v>461</v>
+        <v>481</v>
       </c>
       <c r="D35" t="s">
-        <v>514</v>
+        <v>554</v>
       </c>
       <c r="E35">
         <v>200</v>
@@ -2679,10 +2859,10 @@
         <v>409</v>
       </c>
       <c r="C50" t="s">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="D50" t="s">
-        <v>515</v>
+        <v>555</v>
       </c>
       <c r="E50">
         <v>200</v>
@@ -2696,10 +2876,10 @@
         <v>410</v>
       </c>
       <c r="C51" t="s">
-        <v>463</v>
+        <v>483</v>
       </c>
       <c r="D51" t="s">
-        <v>516</v>
+        <v>556</v>
       </c>
       <c r="E51">
         <v>200</v>
@@ -2713,10 +2893,10 @@
         <v>411</v>
       </c>
       <c r="C52" t="s">
-        <v>464</v>
+        <v>484</v>
       </c>
       <c r="D52" t="s">
-        <v>517</v>
+        <v>557</v>
       </c>
       <c r="E52">
         <v>200</v>
@@ -2730,10 +2910,10 @@
         <v>412</v>
       </c>
       <c r="C53" t="s">
-        <v>465</v>
+        <v>485</v>
       </c>
       <c r="D53" t="s">
-        <v>518</v>
+        <v>558</v>
       </c>
       <c r="E53">
         <v>200</v>
@@ -2747,10 +2927,10 @@
         <v>413</v>
       </c>
       <c r="C54" t="s">
-        <v>466</v>
+        <v>486</v>
       </c>
       <c r="D54" t="s">
-        <v>519</v>
+        <v>559</v>
       </c>
       <c r="E54">
         <v>200</v>
@@ -2764,10 +2944,10 @@
         <v>414</v>
       </c>
       <c r="C55" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="D55" t="s">
-        <v>520</v>
+        <v>560</v>
       </c>
       <c r="E55">
         <v>200</v>
@@ -2781,10 +2961,10 @@
         <v>415</v>
       </c>
       <c r="C56" t="s">
-        <v>468</v>
+        <v>488</v>
       </c>
       <c r="D56" t="s">
-        <v>521</v>
+        <v>561</v>
       </c>
       <c r="E56">
         <v>200</v>
@@ -2798,10 +2978,10 @@
         <v>416</v>
       </c>
       <c r="C57" t="s">
-        <v>469</v>
+        <v>489</v>
       </c>
       <c r="D57" t="s">
-        <v>522</v>
+        <v>562</v>
       </c>
       <c r="E57">
         <v>200</v>
@@ -2815,10 +2995,10 @@
         <v>417</v>
       </c>
       <c r="C58" t="s">
-        <v>470</v>
+        <v>490</v>
       </c>
       <c r="D58" t="s">
-        <v>523</v>
+        <v>563</v>
       </c>
       <c r="E58">
         <v>200</v>
@@ -2832,10 +3012,10 @@
         <v>418</v>
       </c>
       <c r="C59" t="s">
-        <v>471</v>
+        <v>491</v>
       </c>
       <c r="D59" t="s">
-        <v>524</v>
+        <v>564</v>
       </c>
       <c r="E59">
         <v>200</v>
@@ -2849,10 +3029,10 @@
         <v>419</v>
       </c>
       <c r="C60" t="s">
-        <v>472</v>
+        <v>492</v>
       </c>
       <c r="D60" t="s">
-        <v>525</v>
+        <v>565</v>
       </c>
       <c r="E60">
         <v>200</v>
@@ -2866,10 +3046,10 @@
         <v>420</v>
       </c>
       <c r="C61" t="s">
-        <v>473</v>
+        <v>493</v>
       </c>
       <c r="D61" t="s">
-        <v>526</v>
+        <v>566</v>
       </c>
       <c r="E61">
         <v>200</v>
@@ -2883,10 +3063,10 @@
         <v>421</v>
       </c>
       <c r="C62" t="s">
-        <v>474</v>
+        <v>494</v>
       </c>
       <c r="D62" t="s">
-        <v>527</v>
+        <v>567</v>
       </c>
       <c r="E62">
         <v>200</v>
@@ -2900,10 +3080,10 @@
         <v>422</v>
       </c>
       <c r="C63" t="s">
-        <v>475</v>
+        <v>495</v>
       </c>
       <c r="D63" t="s">
-        <v>528</v>
+        <v>568</v>
       </c>
       <c r="E63">
         <v>200</v>
@@ -2967,10 +3147,10 @@
         <v>423</v>
       </c>
       <c r="C74" t="s">
-        <v>476</v>
+        <v>496</v>
       </c>
       <c r="D74" t="s">
-        <v>529</v>
+        <v>569</v>
       </c>
       <c r="E74">
         <v>200</v>
@@ -2984,10 +3164,10 @@
         <v>424</v>
       </c>
       <c r="C75" t="s">
-        <v>477</v>
+        <v>497</v>
       </c>
       <c r="D75" t="s">
-        <v>530</v>
+        <v>570</v>
       </c>
       <c r="E75">
         <v>200</v>
@@ -3001,10 +3181,10 @@
         <v>425</v>
       </c>
       <c r="C76" t="s">
-        <v>478</v>
+        <v>498</v>
       </c>
       <c r="D76" t="s">
-        <v>531</v>
+        <v>571</v>
       </c>
       <c r="E76">
         <v>200</v>
@@ -3018,10 +3198,10 @@
         <v>426</v>
       </c>
       <c r="C77" t="s">
-        <v>479</v>
+        <v>499</v>
       </c>
       <c r="D77" t="s">
-        <v>532</v>
+        <v>572</v>
       </c>
       <c r="E77">
         <v>200</v>
@@ -3035,10 +3215,10 @@
         <v>427</v>
       </c>
       <c r="C78" t="s">
-        <v>480</v>
+        <v>500</v>
       </c>
       <c r="D78" t="s">
-        <v>533</v>
+        <v>573</v>
       </c>
       <c r="E78">
         <v>200</v>
@@ -3052,10 +3232,10 @@
         <v>428</v>
       </c>
       <c r="C79" t="s">
-        <v>481</v>
+        <v>501</v>
       </c>
       <c r="D79" t="s">
-        <v>534</v>
+        <v>574</v>
       </c>
       <c r="E79">
         <v>200</v>
@@ -3069,10 +3249,10 @@
         <v>429</v>
       </c>
       <c r="C80" t="s">
-        <v>482</v>
+        <v>502</v>
       </c>
       <c r="D80" t="s">
-        <v>535</v>
+        <v>575</v>
       </c>
       <c r="E80">
         <v>200</v>
@@ -3171,10 +3351,10 @@
         <v>430</v>
       </c>
       <c r="C98" t="s">
-        <v>483</v>
+        <v>503</v>
       </c>
       <c r="D98" t="s">
-        <v>536</v>
+        <v>576</v>
       </c>
       <c r="E98">
         <v>200</v>
@@ -3303,10 +3483,10 @@
         <v>431</v>
       </c>
       <c r="C122" t="s">
-        <v>484</v>
+        <v>504</v>
       </c>
       <c r="D122" t="s">
-        <v>537</v>
+        <v>577</v>
       </c>
       <c r="E122">
         <v>200</v>
@@ -3320,10 +3500,10 @@
         <v>432</v>
       </c>
       <c r="C123" t="s">
-        <v>485</v>
+        <v>505</v>
       </c>
       <c r="D123" t="s">
-        <v>538</v>
+        <v>578</v>
       </c>
       <c r="E123">
         <v>200</v>
@@ -3337,10 +3517,10 @@
         <v>433</v>
       </c>
       <c r="C124" t="s">
-        <v>486</v>
+        <v>506</v>
       </c>
       <c r="D124" t="s">
-        <v>539</v>
+        <v>579</v>
       </c>
       <c r="E124">
         <v>200</v>
@@ -3354,10 +3534,10 @@
         <v>434</v>
       </c>
       <c r="C125" t="s">
-        <v>487</v>
+        <v>507</v>
       </c>
       <c r="D125" t="s">
-        <v>540</v>
+        <v>580</v>
       </c>
       <c r="E125">
         <v>200</v>
@@ -3471,10 +3651,10 @@
         <v>435</v>
       </c>
       <c r="C146" t="s">
-        <v>488</v>
+        <v>508</v>
       </c>
       <c r="D146" t="s">
-        <v>541</v>
+        <v>581</v>
       </c>
       <c r="E146">
         <v>200</v>
@@ -3488,10 +3668,10 @@
         <v>436</v>
       </c>
       <c r="C147" t="s">
-        <v>489</v>
+        <v>509</v>
       </c>
       <c r="D147" t="s">
-        <v>542</v>
+        <v>582</v>
       </c>
       <c r="E147">
         <v>200</v>
@@ -3505,10 +3685,10 @@
         <v>437</v>
       </c>
       <c r="C148" t="s">
-        <v>490</v>
+        <v>510</v>
       </c>
       <c r="D148" t="s">
-        <v>543</v>
+        <v>583</v>
       </c>
       <c r="E148">
         <v>200</v>
@@ -3522,10 +3702,10 @@
         <v>438</v>
       </c>
       <c r="C149" t="s">
-        <v>491</v>
+        <v>511</v>
       </c>
       <c r="D149" t="s">
-        <v>544</v>
+        <v>584</v>
       </c>
       <c r="E149">
         <v>200</v>
@@ -3539,10 +3719,10 @@
         <v>439</v>
       </c>
       <c r="C150" t="s">
-        <v>492</v>
+        <v>512</v>
       </c>
       <c r="D150" t="s">
-        <v>545</v>
+        <v>585</v>
       </c>
       <c r="E150">
         <v>200</v>
@@ -3556,10 +3736,10 @@
         <v>440</v>
       </c>
       <c r="C151" t="s">
-        <v>493</v>
+        <v>513</v>
       </c>
       <c r="D151" t="s">
-        <v>546</v>
+        <v>586</v>
       </c>
       <c r="E151">
         <v>200</v>
@@ -3573,10 +3753,10 @@
         <v>441</v>
       </c>
       <c r="C152" t="s">
-        <v>494</v>
+        <v>514</v>
       </c>
       <c r="D152" t="s">
-        <v>547</v>
+        <v>587</v>
       </c>
       <c r="E152">
         <v>200</v>
@@ -3782,242 +3962,482 @@
         <v>195</v>
       </c>
     </row>
-    <row r="193" spans="1:1">
+    <row r="193" spans="1:5">
       <c r="A193" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="194" spans="1:1">
+    <row r="194" spans="1:5">
       <c r="A194" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="195" spans="1:1">
+      <c r="B194" t="s">
+        <v>442</v>
+      </c>
+      <c r="C194" t="s">
+        <v>515</v>
+      </c>
+      <c r="D194" t="s">
+        <v>588</v>
+      </c>
+      <c r="E194">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5">
       <c r="A195" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="196" spans="1:1">
+      <c r="B195" t="s">
+        <v>443</v>
+      </c>
+      <c r="C195" t="s">
+        <v>516</v>
+      </c>
+      <c r="D195" t="s">
+        <v>589</v>
+      </c>
+      <c r="E195">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5">
       <c r="A196" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="197" spans="1:1">
+      <c r="B196" t="s">
+        <v>444</v>
+      </c>
+      <c r="C196" t="s">
+        <v>517</v>
+      </c>
+      <c r="D196" t="s">
+        <v>590</v>
+      </c>
+      <c r="E196">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5">
       <c r="A197" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="198" spans="1:1">
+      <c r="B197" t="s">
+        <v>445</v>
+      </c>
+      <c r="C197" t="s">
+        <v>518</v>
+      </c>
+      <c r="D197" t="s">
+        <v>591</v>
+      </c>
+      <c r="E197">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5">
       <c r="A198" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="199" spans="1:1">
+      <c r="B198" t="s">
+        <v>446</v>
+      </c>
+      <c r="C198" t="s">
+        <v>519</v>
+      </c>
+      <c r="D198" t="s">
+        <v>592</v>
+      </c>
+      <c r="E198">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5">
       <c r="A199" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="200" spans="1:1">
+      <c r="B199" t="s">
+        <v>447</v>
+      </c>
+      <c r="C199" t="s">
+        <v>520</v>
+      </c>
+      <c r="D199" t="s">
+        <v>593</v>
+      </c>
+      <c r="E199">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5">
       <c r="A200" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="201" spans="1:1">
+      <c r="B200" t="s">
+        <v>448</v>
+      </c>
+      <c r="C200" t="s">
+        <v>521</v>
+      </c>
+      <c r="D200" t="s">
+        <v>594</v>
+      </c>
+      <c r="E200">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5">
       <c r="A201" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="202" spans="1:1">
+      <c r="B201" t="s">
+        <v>449</v>
+      </c>
+      <c r="C201" t="s">
+        <v>522</v>
+      </c>
+      <c r="D201" t="s">
+        <v>595</v>
+      </c>
+      <c r="E201">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5">
       <c r="A202" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="203" spans="1:1">
+      <c r="B202" t="s">
+        <v>450</v>
+      </c>
+      <c r="C202" t="s">
+        <v>523</v>
+      </c>
+      <c r="D202" t="s">
+        <v>596</v>
+      </c>
+      <c r="E202">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5">
       <c r="A203" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="204" spans="1:1">
+      <c r="B203" t="s">
+        <v>451</v>
+      </c>
+      <c r="C203" t="s">
+        <v>524</v>
+      </c>
+      <c r="D203" t="s">
+        <v>597</v>
+      </c>
+      <c r="E203">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5">
       <c r="A204" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="205" spans="1:1">
+    <row r="205" spans="1:5">
       <c r="A205" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="206" spans="1:1">
+    <row r="206" spans="1:5">
       <c r="A206" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="207" spans="1:1">
+    <row r="207" spans="1:5">
       <c r="A207" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="208" spans="1:1">
+    <row r="208" spans="1:5">
       <c r="A208" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="209" spans="1:1">
+    <row r="209" spans="1:5">
       <c r="A209" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="210" spans="1:1">
+    <row r="210" spans="1:5">
       <c r="A210" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="211" spans="1:1">
+    <row r="211" spans="1:5">
       <c r="A211" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="212" spans="1:1">
+    <row r="212" spans="1:5">
       <c r="A212" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="213" spans="1:1">
+    <row r="213" spans="1:5">
       <c r="A213" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="214" spans="1:1">
+    <row r="214" spans="1:5">
       <c r="A214" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="215" spans="1:1">
+    <row r="215" spans="1:5">
       <c r="A215" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="216" spans="1:1">
+    <row r="216" spans="1:5">
       <c r="A216" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="217" spans="1:1">
+    <row r="217" spans="1:5">
       <c r="A217" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="218" spans="1:1">
+    <row r="218" spans="1:5">
       <c r="A218" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="219" spans="1:1">
+      <c r="B218" t="s">
+        <v>452</v>
+      </c>
+      <c r="C218" t="s">
+        <v>525</v>
+      </c>
+      <c r="D218" t="s">
+        <v>598</v>
+      </c>
+      <c r="E218">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5">
       <c r="A219" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="220" spans="1:1">
+      <c r="B219" t="s">
+        <v>453</v>
+      </c>
+      <c r="C219" t="s">
+        <v>526</v>
+      </c>
+      <c r="D219" t="s">
+        <v>599</v>
+      </c>
+      <c r="E219">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5">
       <c r="A220" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="221" spans="1:1">
+      <c r="B220" t="s">
+        <v>454</v>
+      </c>
+      <c r="C220" t="s">
+        <v>527</v>
+      </c>
+      <c r="D220" t="s">
+        <v>600</v>
+      </c>
+      <c r="E220">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5">
       <c r="A221" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="222" spans="1:1">
+      <c r="B221" t="s">
+        <v>455</v>
+      </c>
+      <c r="C221" t="s">
+        <v>528</v>
+      </c>
+      <c r="D221" t="s">
+        <v>601</v>
+      </c>
+      <c r="E221">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5">
       <c r="A222" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="223" spans="1:1">
+      <c r="B222" t="s">
+        <v>456</v>
+      </c>
+      <c r="C222" t="s">
+        <v>529</v>
+      </c>
+      <c r="D222" t="s">
+        <v>602</v>
+      </c>
+      <c r="E222">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5">
       <c r="A223" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="224" spans="1:1">
+      <c r="B223" t="s">
+        <v>457</v>
+      </c>
+      <c r="C223" t="s">
+        <v>530</v>
+      </c>
+      <c r="D223" t="s">
+        <v>603</v>
+      </c>
+      <c r="E223">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5">
       <c r="A224" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="225" spans="1:1">
+      <c r="B224" t="s">
+        <v>458</v>
+      </c>
+      <c r="C224" t="s">
+        <v>531</v>
+      </c>
+      <c r="D224" t="s">
+        <v>604</v>
+      </c>
+      <c r="E224">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5">
       <c r="A225" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="226" spans="1:1">
+      <c r="B225" t="s">
+        <v>459</v>
+      </c>
+      <c r="C225" t="s">
+        <v>532</v>
+      </c>
+      <c r="D225" t="s">
+        <v>605</v>
+      </c>
+      <c r="E225">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5">
       <c r="A226" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="227" spans="1:1">
+      <c r="B226" t="s">
+        <v>460</v>
+      </c>
+      <c r="C226" t="s">
+        <v>533</v>
+      </c>
+      <c r="D226" t="s">
+        <v>606</v>
+      </c>
+      <c r="E226">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5">
       <c r="A227" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="228" spans="1:1">
+      <c r="B227" t="s">
+        <v>461</v>
+      </c>
+      <c r="C227" t="s">
+        <v>534</v>
+      </c>
+      <c r="D227" t="s">
+        <v>607</v>
+      </c>
+      <c r="E227">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5">
       <c r="A228" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="229" spans="1:1">
+    <row r="229" spans="1:5">
       <c r="A229" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="230" spans="1:1">
+    <row r="230" spans="1:5">
       <c r="A230" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="231" spans="1:1">
+    <row r="231" spans="1:5">
       <c r="A231" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="232" spans="1:1">
+    <row r="232" spans="1:5">
       <c r="A232" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="233" spans="1:1">
+    <row r="233" spans="1:5">
       <c r="A233" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="234" spans="1:1">
+    <row r="234" spans="1:5">
       <c r="A234" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="235" spans="1:1">
+    <row r="235" spans="1:5">
       <c r="A235" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="236" spans="1:1">
+    <row r="236" spans="1:5">
       <c r="A236" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="237" spans="1:1">
+    <row r="237" spans="1:5">
       <c r="A237" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="238" spans="1:1">
+    <row r="238" spans="1:5">
       <c r="A238" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="239" spans="1:1">
+    <row r="239" spans="1:5">
       <c r="A239" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="240" spans="1:1">
+    <row r="240" spans="1:5">
       <c r="A240" t="s">
         <v>243</v>
       </c>
@@ -4773,84 +5193,84 @@
   <sheetData>
     <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
-        <v>572</v>
+        <v>632</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>548</v>
+        <v>608</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>549</v>
+        <v>609</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>550</v>
+        <v>610</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>551</v>
+        <v>611</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>552</v>
+        <v>612</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>553</v>
+        <v>613</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>554</v>
+        <v>614</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>555</v>
+        <v>615</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>556</v>
+        <v>616</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>557</v>
+        <v>617</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>558</v>
+        <v>618</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>559</v>
+        <v>619</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>560</v>
+        <v>620</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>561</v>
+        <v>621</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>562</v>
+        <v>622</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>563</v>
+        <v>623</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>564</v>
+        <v>624</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>565</v>
+        <v>625</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>566</v>
+        <v>626</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>567</v>
+        <v>627</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>568</v>
+        <v>628</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>569</v>
+        <v>629</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>570</v>
+        <v>630</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>571</v>
+        <v>631</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="2" customFormat="1">
       <c r="A2" s="1" t="s">
-        <v>573</v>
+        <v>633</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>389</v>
@@ -4885,7 +5305,7 @@
     </row>
     <row r="3" spans="1:25">
       <c r="A3" s="1" t="s">
-        <v>574</v>
+        <v>634</v>
       </c>
       <c r="B3" t="s">
         <v>399</v>
@@ -4920,7 +5340,7 @@
     </row>
     <row r="4" spans="1:25" s="2" customFormat="1">
       <c r="A4" s="1" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>409</v>
@@ -4967,7 +5387,7 @@
     </row>
     <row r="5" spans="1:25">
       <c r="A5" s="1" t="s">
-        <v>576</v>
+        <v>636</v>
       </c>
       <c r="B5" t="s">
         <v>423</v>
@@ -4993,7 +5413,7 @@
     </row>
     <row r="6" spans="1:25" s="2" customFormat="1">
       <c r="A6" s="1" t="s">
-        <v>577</v>
+        <v>637</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>430</v>
@@ -5001,7 +5421,7 @@
     </row>
     <row r="7" spans="1:25">
       <c r="A7" s="1" t="s">
-        <v>578</v>
+        <v>638</v>
       </c>
       <c r="B7" t="s">
         <v>431</v>
@@ -5018,7 +5438,7 @@
     </row>
     <row r="8" spans="1:25" s="2" customFormat="1">
       <c r="A8" s="1" t="s">
-        <v>579</v>
+        <v>639</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>435</v>
@@ -5044,47 +5464,107 @@
     </row>
     <row r="9" spans="1:25">
       <c r="A9" s="1" t="s">
-        <v>580</v>
+        <v>640</v>
       </c>
     </row>
     <row r="10" spans="1:25" s="2" customFormat="1">
       <c r="A10" s="1" t="s">
-        <v>581</v>
+        <v>641</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="1" t="s">
-        <v>582</v>
+        <v>642</v>
+      </c>
+      <c r="B11" t="s">
+        <v>452</v>
+      </c>
+      <c r="C11" t="s">
+        <v>453</v>
+      </c>
+      <c r="D11" t="s">
+        <v>454</v>
+      </c>
+      <c r="E11" t="s">
+        <v>455</v>
+      </c>
+      <c r="F11" t="s">
+        <v>456</v>
+      </c>
+      <c r="G11" t="s">
+        <v>457</v>
+      </c>
+      <c r="H11" t="s">
+        <v>458</v>
+      </c>
+      <c r="I11" t="s">
+        <v>459</v>
+      </c>
+      <c r="J11" t="s">
+        <v>460</v>
+      </c>
+      <c r="K11" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="12" spans="1:25" s="2" customFormat="1">
       <c r="A12" s="1" t="s">
-        <v>583</v>
+        <v>643</v>
       </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="1" t="s">
-        <v>584</v>
+        <v>644</v>
       </c>
     </row>
     <row r="14" spans="1:25" s="2" customFormat="1">
       <c r="A14" s="1" t="s">
-        <v>585</v>
+        <v>645</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" s="1" t="s">
-        <v>586</v>
+        <v>646</v>
       </c>
     </row>
     <row r="16" spans="1:25" s="2" customFormat="1">
       <c r="A16" s="1" t="s">
-        <v>587</v>
+        <v>647</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="1" t="s">
-        <v>588</v>
+        <v>648</v>
       </c>
     </row>
   </sheetData>
@@ -5097,323 +5577,1317 @@
   <dimension ref="A1:Y17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="24" width="5.7109375" customWidth="1"/>
+    <col min="1" max="9" width="3.7109375" customWidth="1"/>
+    <col min="10" max="24" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
-        <v>572</v>
+        <v>632</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>548</v>
+        <v>608</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>549</v>
+        <v>609</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>550</v>
+        <v>610</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>551</v>
+        <v>611</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>552</v>
+        <v>612</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>553</v>
+        <v>613</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>554</v>
+        <v>614</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>555</v>
+        <v>615</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>556</v>
+        <v>616</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>557</v>
+        <v>617</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>558</v>
+        <v>618</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>559</v>
+        <v>619</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>560</v>
+        <v>620</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>561</v>
+        <v>621</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>562</v>
+        <v>622</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>563</v>
+        <v>623</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>564</v>
+        <v>624</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>565</v>
+        <v>625</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>566</v>
+        <v>626</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>567</v>
+        <v>627</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>568</v>
+        <v>628</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>569</v>
+        <v>629</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>570</v>
+        <v>630</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>571</v>
+        <v>631</v>
       </c>
     </row>
     <row r="2" spans="1:25">
       <c r="A2" s="1" t="s">
-        <v>573</v>
+        <v>633</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X2" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y2" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="3" spans="1:25">
       <c r="A3" s="1" t="s">
-        <v>574</v>
+        <v>634</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="4" spans="1:25">
       <c r="A4" s="1" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X4" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y4" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="5" spans="1:25">
       <c r="A5" s="1" t="s">
-        <v>576</v>
+        <v>636</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X5" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y5" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="6" spans="1:25">
       <c r="A6" s="1" t="s">
-        <v>577</v>
+        <v>637</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>589</v>
+        <v>649</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X6" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y6" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="7" spans="1:25">
       <c r="A7" s="1" t="s">
-        <v>578</v>
+        <v>638</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X7" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y7" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="8" spans="1:25">
       <c r="A8" s="1" t="s">
-        <v>579</v>
+        <v>639</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>575</v>
+        <v>635</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X8" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y8" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="9" spans="1:25">
       <c r="A9" s="1" t="s">
-        <v>580</v>
+        <v>640</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X9" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y9" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="10" spans="1:25">
       <c r="A10" s="1" t="s">
-        <v>581</v>
+        <v>641</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X10" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y10" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="1" t="s">
-        <v>582</v>
+        <v>642</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X11" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y11" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="12" spans="1:25">
       <c r="A12" s="1" t="s">
-        <v>583</v>
+        <v>643</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y12" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="1" t="s">
-        <v>584</v>
+        <v>644</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X13" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y13" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="14" spans="1:25">
       <c r="A14" s="1" t="s">
-        <v>585</v>
+        <v>645</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X14" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="15" spans="1:25">
       <c r="A15" s="1" t="s">
-        <v>586</v>
+        <v>646</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X15" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y15" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="16" spans="1:25">
       <c r="A16" s="1" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
+        <v>647</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X16" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y16" s="4" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25">
       <c r="A17" s="1" t="s">
-        <v>588</v>
+        <v>648</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="N17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="R17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="S17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="T17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="U17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="V17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="W17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="X17" s="4" t="s">
+        <v>649</v>
+      </c>
+      <c r="Y17" s="4" t="s">
+        <v>649</v>
       </c>
     </row>
   </sheetData>

</xml_diff>